<commit_message>
feat(landing): home pública rubro-adaptativa con demo en vivo
/ deja de redirigir siempre: muestra una landing pública (redirige a dashboard
solo si hay sesión). Héroe que se adapta al rubro (Kiosco/Carnicería/Servicios/
Atmosféricos/Préstamos) con un mini-POS interactivo + sección antes/después +
pricing en USD cobrado al dólar MEP. Middleware: '/' pasa a ser ruta pública.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -2315,20 +2315,24 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Landing page pública (hoy / redirige al dashboard)</t>
+          <t>Landing page pública (rubro-adaptativa + demo en vivo)</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>/ pública (redirige a dashboard si hay sesión); demo POS interactivo por rubro + antes/después + pricing al MEP</t>
+        </is>
+      </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
           <t>2026-06-20</t>

</xml_diff>

<commit_message>
roadmap: marca landing y legal como Hecho + agrega verticales por versión
- Landing pública y Términos+Privacidad pasan a "Hecho".
- Nueva sección "Versiones / Verticales" con los pendientes del dueño: mejorar
  login, Gesto Balanza funcional, Gesto Food (POS propio), Gesto Servicios
  (boletas + simplificar UI), Gesto Atmosféricos (historial, agenda, pedidos a
  futuro, arreglar Maps).
- Regenera roadmap-gesto.xlsx (fecha 2026-06-21).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SaaS de gestión comercial multi-tenant · Actualizado 2026-06-20 · Editá la columna Estado y la fecha al cerrar cada tarea</t>
+          <t>SaaS de gestión comercial multi-tenant · Actualizado 2026-06-21 · Editá la columna Estado y la fecha al cerrar cada tarea</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       <c r="F21" s="6" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       <c r="F28" s="6" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       <c r="F30" s="6" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       <c r="F31" s="6" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       <c r="F37" s="6" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       <c r="F39" s="6" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       <c r="F40" s="6" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       <c r="F41" s="6" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       <c r="F42" s="6" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
       <c r="F43" s="6" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       <c r="F45" s="6" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
       <c r="F46" s="6" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       <c r="F47" s="6" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       <c r="F48" s="6" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       <c r="F49" s="6" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2315,12 +2315,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Landing page pública (rubro-adaptativa + demo en vivo)</t>
+          <t>Landing page pública (adaptativa por versión + demo en vivo)</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -2330,12 +2330,12 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>/ pública (redirige a dashboard si hay sesión); demo POS interactivo por rubro + antes/después + pricing al MEP</t>
+          <t>v3 'de oficio' LIVE: switcher de versiones auto-rotativo, demo POS con ticket de papel, foto real + captura de Gesto en celular, antes/después, FAQ, pricing al MEP, paleta terracota (sin neón), responsive mobile. Login rediseñado (split de marca)</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>Requerido para cobrar con MP / Ley 25.326</t>
+          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox de aceptación en signup. Responsable: Faro Sistemas (nombre comercial de Tomás de Sousa, persona física). FALTA: completar placeholders [CUIT/domicilio/email/jurisdicción] + revisión de un abogado</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       <c r="F60" s="6" t="inlineStr"/>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       <c r="F61" s="6" t="inlineStr"/>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       <c r="F65" s="6" t="inlineStr"/>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3138,28 +3138,32 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Gestión de mesas (Gesto Food)</t>
+          <t>Mejorar login/registro: sumarle contenido útil (hoy se siente vacío)</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F81" s="6" t="inlineStr"/>
+          <t>En progreso</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>Split de marca ya hecho; falta valor real que sume</t>
+        </is>
+      </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3169,17 +3173,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Integración balanza digital (Gesto Balanza)</t>
+          <t>Gesto Balanza funcional: integración con balanza digital + venta por peso</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
@@ -3187,10 +3191,14 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F82" s="6" t="inlineStr"/>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>Hoy figura 'próximamente'; armarla de verdad para que funcione con balanzas</t>
+        </is>
+      </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3208,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Modificadores por ítem en POS (extras, variantes)</t>
+          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -3218,10 +3226,14 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F83" s="6" t="inlineStr"/>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>Hoy figura 'próximamente'</t>
+        </is>
+      </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3231,17 +3243,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>App mobile nativa con Capacitor (offline first)</t>
+          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
@@ -3249,10 +3261,14 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F84" s="6" t="inlineStr"/>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>La interfaz es muy compleja; hacerla simple y funcional</t>
+        </is>
+      </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3262,17 +3278,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Notificaciones push (stock, pedidos)</t>
+          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
@@ -3280,10 +3296,14 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F85" s="6" t="inlineStr"/>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>La función de Maps no toma bien las direcciones</t>
+        </is>
+      </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3318,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
+          <t>Modificadores por ítem en POS (extras, variantes)</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3314,7 +3334,7 @@
       <c r="F86" s="6" t="inlineStr"/>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3349,7 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+          <t>App mobile nativa con Capacitor (offline first)</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3345,17 +3365,110 @@
       <c r="F87" s="6" t="inlineStr"/>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Roadmap v2</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>Notificaciones push (stock, pedidos)</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr"/>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Roadmap v2</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr"/>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Roadmap v2</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G87"/>
+  <autoFilter ref="A4:G90"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G87">
+  <conditionalFormatting sqref="A5:G90">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3367,10 +3480,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3384,7 +3497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3423,7 +3536,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$87,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$90,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3438,7 +3551,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$87,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$90,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3453,7 +3566,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$87,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$90,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3468,7 +3581,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$87)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$90)</f>
         <v/>
       </c>
     </row>
@@ -3496,11 +3609,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A11,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A11,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -3511,11 +3624,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A12,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A12,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -3526,11 +3639,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A13,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A13,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -3541,11 +3654,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A14,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A14,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -3556,11 +3669,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A15,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A15,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -3571,11 +3684,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A16,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A16,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -3586,11 +3699,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A17,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A17,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -3601,11 +3714,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A18,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A18,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -3616,11 +3729,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A19,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A19,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -3631,11 +3744,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A20,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A20,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -3646,11 +3759,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A21,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A21,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -3661,11 +3774,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A22,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A22,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -3676,11 +3789,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A23,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A23,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -3691,11 +3804,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A24,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A24,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -3706,11 +3819,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A25,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A25,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -3721,11 +3834,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A26,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A26,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -3736,11 +3849,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A27,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A27,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -3751,26 +3864,41 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A28,Roadmap!$E$5:$E$87,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A28,Roadmap!$E$5:$E$90,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A28)-B28</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Versiones / Verticales</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A29,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <v/>
+      </c>
+      <c r="C29">
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A29)-B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Roadmap v2</t>
         </is>
       </c>
-      <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A29,Roadmap!$E$5:$E$87,"Hecho")</f>
-        <v/>
-      </c>
-      <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$87,A29)-B29</f>
+      <c r="B30">
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A30,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <v/>
+      </c>
+      <c r="C30">
+        <f>COUNTIFS(Roadmap!$B$5:$B$90,A30)-B30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
POS: soporte de lector de códigos USB (Enter agrega) + roadmap
- El buscador del POS (minorista y mayorista) ahora agrega el producto al apretar
  Enter: coincidencia exacta por código de barras (lo que entrega el lector USB
  tipo supermercado) y limpia para el siguiente scan. No requiere permisos.
- Roadmap: lector USB = Hecho; Gesto Servicios = En progreso (form simplificado
  hecho, boletas en curso). Regenera roadmap-gesto.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Cuenta Corriente</t>
+          <t>Ventas / POS</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Movimientos + registrar pago + saldo en tiempo real</t>
+          <t>Lector de códigos USB en POS desktop (Enter agrega el producto escaneado)</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>registrarPago atómico FOR UPDATE</t>
+          <t>Minorista + mayorista; el lector tipo supermercado escribe el código y Enter lo suma al carrito</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Reversión de movimientos (transacción atómica)</t>
+          <t>Movimientos + registrar pago + saldo en tiempo real</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>motivo obligatorio</t>
+          <t>registrarPago atómico FOR UPDATE</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Reportes</t>
+          <t>Cuenta Corriente</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>KPIs por período + ranking top productos + métodos de pago</t>
+          <t>Reversión de movimientos (transacción atómica)</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>ventana de tiempo unificada</t>
+          <t>motivo obligatorio</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Exportar a CSV</t>
+          <t>KPIs por período + ranking top productos + métodos de pago</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1672,7 +1672,11 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>ventana de tiempo unificada</t>
+        </is>
+      </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -1685,12 +1689,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Presupuestos</t>
+          <t>Reportes</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>CRUD + PDF + estados + numeración atómica</t>
+          <t>Exportar a CSV</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1703,11 +1707,7 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>db.transaction</t>
-        </is>
-      </c>
+      <c r="F38" s="6" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Plantillas de servicios (guardar/listar/usar)</t>
+          <t>CRUD + PDF + estados + numeración atómica</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1738,7 +1738,11 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>db.transaction</t>
+        </is>
+      </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -1751,12 +1755,12 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Proveedores / Pedidos</t>
+          <t>Presupuestos</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>CRUD proveedores (markup, selector de país)</t>
+          <t>Plantillas de servicios (guardar/listar/usar)</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1787,7 +1791,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Pedidos a proveedor (WhatsApp + recepción con ajuste de stock)</t>
+          <t>CRUD proveedores (markup, selector de país)</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1813,12 +1817,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Configuración / Equipo</t>
+          <t>Proveedores / Pedidos</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Datos fiscales + canales + conectar/desconectar Mercado Pago</t>
+          <t>Pedidos a proveedor (WhatsApp + recepción con ajuste de stock)</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1849,7 +1853,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Equipo: invitar por email, editar rol, eliminar</t>
+          <t>Datos fiscales + canales + conectar/desconectar Mercado Pago</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1880,7 +1884,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Control de acceso por rol (requireAdmin, route group)</t>
+          <t>Equipo: invitar por email, editar rol, eliminar</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1893,11 +1897,7 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>empleado solo POS+Historial+Productos</t>
-        </is>
-      </c>
+      <c r="F44" s="6" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -1910,12 +1910,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>UX / Diseño</t>
+          <t>Configuración / Equipo</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Design System Brasas v2 (paleta cálida + grain + gradientes)</t>
+          <t>Control de acceso por rol (requireAdmin, route group)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1928,7 +1928,11 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>empleado solo POS+Historial+Productos</t>
+        </is>
+      </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -1946,7 +1950,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Sidebar + mobile bottom nav con FAB Vender</t>
+          <t>Design System Brasas v2 (paleta cálida + grain + gradientes)</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1977,7 +1981,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Skeleton loaders (7 rutas)</t>
+          <t>Sidebar + mobile bottom nav con FAB Vender</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2008,7 +2012,7 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Command palette ⌘K</t>
+          <t>Skeleton loaders (7 rutas)</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2039,17 +2043,17 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Dark / light toggle</t>
+          <t>Command palette ⌘K</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr"/>
@@ -2065,29 +2069,25 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Negocio SaaS</t>
+          <t>UX / Diseño</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>4 planes + Mercado Pago preapproval + webhook activación/suspensión</t>
+          <t>Dark / light toggle</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>src/lib/planes.ts</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr"/>
       <c r="G50" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Cobro por transferencia (panel admin + aviso cliente + comprobante por email)</t>
+          <t>4 planes + Mercado Pago preapproval + webhook activación/suspensión</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>Activación manual 1-click; /admin/suscripciones; emails salen al cargar RESEND_API_KEY</t>
+          <t>src/lib/planes.ts</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
@@ -2140,22 +2140,22 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Cobro automático MP/Mobbex (CUIT Monotributo + cuenta)</t>
+          <t>Cobro por transferencia (panel admin + aviso cliente + comprobante por email)</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Bloqueado: falta CUIT + cuenta. Mientras tanto se cobra por transferencia</t>
+          <t>Activación manual 1-click; /admin/suscripciones; emails salen al cargar RESEND_API_KEY</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Panel super-admin (gestionar tenants, métricas cross-tenant)</t>
+          <t>Cobro automático MP/Mobbex (CUIT Monotributo + cuenta)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>Panel /admin/suscripciones operativo; faltan métricas cross-tenant</t>
+          <t>Bloqueado: falta CUIT + cuenta. Mientras tanto se cobra por transferencia</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -2210,22 +2210,22 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Catálogo global cross-tenant</t>
+          <t>Panel super-admin (gestionar tenants, métricas cross-tenant)</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Necesita OK explícito antes de implementar</t>
+          <t>Panel /admin/suscripciones operativo; faltan métricas cross-tenant</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -2240,17 +2240,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Lanzamiento (bloqueante)</t>
+          <t>Negocio SaaS</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Dominio propio (ej: usegesto.app)</t>
+          <t>Catálogo global cross-tenant</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>URL actual no es presentable</t>
+          <t>Necesita OK explícito antes de implementar</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>SMTP con Resend (invitación, bienvenida, reset con branding)</t>
+          <t>Dominio propio (ej: usegesto.app)</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>Cron listo; falta RESEND_API_KEY en Vercel (rotar la vieja)</t>
+          <t>URL actual no es presentable</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Landing page pública (adaptativa por versión + demo en vivo)</t>
+          <t>SMTP con Resend (invitación, bienvenida, reset con branding)</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2325,12 +2325,12 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>v3 'de oficio' LIVE: switcher de versiones auto-rotativo, demo POS con ticket de papel, foto real + captura de Gesto en celular, antes/después, FAQ, pricing al MEP, paleta terracota (sin neón), responsive mobile. Login rediseñado (split de marca)</t>
+          <t>Cron listo; falta RESEND_API_KEY en Vercel (rotar la vieja)</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>PWA manifest + iconos (192/512, apple-touch-icon)</t>
+          <t>Landing page pública (adaptativa por versión + demo en vivo)</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2360,12 +2360,12 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>POS se usa en tablet/celular</t>
+          <t>v3 'de oficio' LIVE: switcher de versiones auto-rotativo, demo POS con ticket de papel, foto real + captura de Gesto en celular, antes/después, FAQ, pricing al MEP, paleta terracota (sin neón), responsive mobile. Login rediseñado (split de marca)</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Términos de servicio + Política de privacidad</t>
+          <t>PWA manifest + iconos (192/512, apple-touch-icon)</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox de aceptación en signup. Responsable: Faro Sistemas (nombre comercial de Tomás de Sousa, persona física). FALTA: completar placeholders [CUIT/domicilio/email/jurisdicción] + revisión de un abogado</t>
+          <t>POS se usa en tablet/celular</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -2415,17 +2415,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Calidad / Seguridad</t>
+          <t>Lanzamiento (bloqueante)</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Bugs críticos corregidos (stock al vender, numeración, loop /planes)</t>
+          <t>Términos de servicio + Política de privacidad</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -2433,7 +2433,11 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr"/>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox de aceptación en signup. Responsable: Faro Sistemas (nombre comercial de Tomás de Sousa, persona física). FALTA: completar placeholders [CUIT/domicilio/email/jurisdicción] + revisión de un abogado</t>
+        </is>
+      </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2451,7 +2455,7 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>ConfirmDialog reutilizable (reemplaza window.confirm en 9 comp.)</t>
+          <t>Bugs críticos corregidos (stock al vender, numeración, loop /planes)</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -2482,7 +2486,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Verificar firma de webhook MP</t>
+          <t>ConfirmDialog reutilizable (reemplaza window.confirm en 9 comp.)</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2495,11 +2499,7 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>Firma HMAC timing-safe + fail-closed en prod; cargar MP_WEBHOOK_SECRET en Vercel</t>
-        </is>
-      </c>
+      <c r="F62" s="6" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Auditoría de seguridad E2E + fixes (IDOR token MP, recibirPedido, escalación de rol, OAuth state, crons fail-closed, escape de emails)</t>
+          <t>Verificar firma de webhook MP</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>Guard test anti-omisión de byTenant; ver project_gesto_seguridad. RLS no protege capa app (byTenant única defensa)</t>
+          <t>Firma HMAC timing-safe + fail-closed en prod; cargar MP_WEBHOOK_SECRET en Vercel</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
@@ -2552,22 +2552,22 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Rate limiting en auth (login/signup)</t>
+          <t>Auditoría de seguridad E2E + fixes (IDOR token MP, recibirPedido, escalación de rol, OAuth state, crons fail-closed, escape de emails)</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>ej: @upstash/ratelimit</t>
+          <t>Guard test anti-omisión de byTenant; ver project_gesto_seguridad. RLS no protege capa app (byTenant única defensa)</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Tests de integración (flows de venta y producto)</t>
+          <t>Rate limiting en auth (login/signup)</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -2600,7 +2600,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr"/>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>ej: @upstash/ratelimit</t>
+        </is>
+      </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2618,7 +2622,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Export de datos (CSV ventas / inventario)</t>
+          <t>Tests de integración (flows de venta y producto)</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2631,11 +2635,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>Que el cliente no sienta lock-in</t>
-        </is>
-      </c>
+      <c r="F66" s="6" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Facturación AFIP (Tusfacturas.app, A/B)</t>
+          <t>Export de datos (CSV ventas / inventario)</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>Bloqueante segmento servicios/mayorista</t>
+          <t>Que el cliente no sienta lock-in</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
@@ -2688,12 +2688,12 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Historial de auditoría básico (quién creó/modificó)</t>
+          <t>Facturación AFIP (Tusfacturas.app, A/B)</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>Mínimo en productos y ventas</t>
+          <t>Bloqueante segmento servicios/mayorista</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
@@ -2718,17 +2718,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Legal / Fiscal</t>
+          <t>Calidad / Seguridad</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>CUIT + Monotributo (o Responsable Inscripto)</t>
+          <t>Historial de auditoría básico (quién creó/modificó)</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>Bloquea cobrar en regla; ojo el tope anual de Monotributo con ingresos SaaS recurrentes</t>
+          <t>Mínimo en productos y ventas</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -2758,12 +2758,12 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Registro de bases de datos ante la AAIP (Ley 25.326)</t>
+          <t>CUIT + Monotributo (o Responsable Inscripto)</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>Sos responsable de la PII de los clientes y de SUS clientes</t>
+          <t>Bloquea cobrar en regla; ojo el tope anual de Monotributo con ingresos SaaS recurrentes</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Botón de baja + arrepentimiento de suscripción (Res. 424/2020)</t>
+          <t>Registro de bases de datos ante la AAIP (Ley 25.326)</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>Cancelación online fácil y visible; ya existe cancelarSuscripcion</t>
+          <t>Sos responsable de la PII de los clientes y de SUS clientes</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Cláusulas de transferencia internacional de datos</t>
+          <t>Botón de baja + arrepentimiento de suscripción (Res. 424/2020)</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>Datos en AWS us-east-1; Ley 25.326 exige resguardos (EE.UU. no es país adecuado por defecto)</t>
+          <t>Cancelación online fácil y visible; ya existe cancelarSuscripcion</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Estructura societaria (SAS) + acuerdo escrito con socio</t>
+          <t>Cláusulas de transferencia internacional de datos</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
@@ -2878,7 +2878,7 @@
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>Separa patrimonio del riesgo; formaliza la participación de Facu</t>
+          <t>Datos en AWS us-east-1; Ley 25.326 exige resguardos (EE.UU. no es país adecuado por defecto)</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Contrato de servicio / SLA con clientes</t>
+          <t>Estructura societaria (SAS) + acuerdo escrito con socio</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>Dueño de los datos (el cliente), uptime, soporte, límite de responsabilidad</t>
+          <t>Separa patrimonio del riesgo; formaliza la participación de Facu</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -2928,17 +2928,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Infra / Escalado</t>
+          <t>Legal / Fiscal</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Vercel Pro + Supabase Pro</t>
+          <t>Contrato de servicio / SLA con clientes</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>Vercel Hobby es no comercial; Supabase Free se pausa a los 7 días. Bloquea producción real</t>
+          <t>Dueño de los datos (el cliente), uptime, soporte, límite de responsabilidad</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
@@ -2968,12 +2968,12 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Backups diarios + PITR + probar un restore</t>
+          <t>Vercel Pro + Supabase Pro</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>Un backup sin restore probado no es un backup</t>
+          <t>Vercel Hobby es no comercial; Supabase Free se pausa a los 7 días. Bloquea producción real</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Monitoreo: activar Sentry + uptime check</t>
+          <t>Backups diarios + PITR + probar un restore</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>SENTRY_DSN ya está en el build, falta activarlo + un cron canario</t>
+          <t>Un backup sin restore probado no es un backup</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Email deliverability: dominio + SPF/DKIM/DMARC (Resend)</t>
+          <t>Monitoreo: activar Sentry + uptime check</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>Si no, comprobantes y facturas caen en spam</t>
+          <t>SENTRY_DSN ya está en el build, falta activarlo + un cron canario</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Encriptar tokens MP del negocio at-rest</t>
+          <t>Email deliverability: dominio + SPF/DKIM/DMARC (Resend)</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>Hoy en texto plano en tenants (hallazgo de seguridad #9)</t>
+          <t>Si no, comprobantes y facturas caen en spam</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -3103,12 +3103,12 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Backlog / Ideas</t>
+          <t>Infra / Escalado</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Consultor de precios para cliente final (pantalla pública con QR)</t>
+          <t>Encriptar tokens MP del negocio at-rest</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>Diferenciador único; ruta /p/[tenantSlug]</t>
+          <t>Hoy en texto plano en tenants (hallazgo de seguridad #9)</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Versiones / Verticales</t>
+          <t>Backlog / Ideas</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Mejorar login/registro: sumarle contenido útil (hoy se siente vacío)</t>
+          <t>Consultor de precios para cliente final (pantalla pública con QR)</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -3153,12 +3153,12 @@
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>Split de marca ya hecho; falta valor real que sume</t>
+          <t>Diferenciador único; ruta /p/[tenantSlug]</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -3178,22 +3178,22 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Gesto Balanza funcional: integración con balanza digital + venta por peso</t>
+          <t>Mejorar login/registro: sumarle contenido útil (hoy se siente vacío)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>Hoy figura 'próximamente'; armarla de verdad para que funcione con balanzas</t>
+          <t>Split de marca ya hecho; falta valor real que sume</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
+          <t>Gesto Balanza funcional: integración con balanza digital + venta por peso</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>Hoy figura 'próximamente'</t>
+          <t>Hoy figura 'próximamente'; armarla de verdad para que funcione con balanzas</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
+          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>La interfaz es muy compleja; hacerla simple y funcional</t>
+          <t>Hoy figura 'próximamente'</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
+          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>La función de Maps no toma bien las direcciones</t>
+          <t>Formulario de presupuesto SIMPLIFICADO (hecho: cliente unificado, mano de obra directa, opciones plegables); boletas = comprobante de cobro no fiscal (al cobrar un presupuesto + boleta directa) en curso</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -3313,17 +3313,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Modificadores por ítem en POS (extras, variantes)</t>
+          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
@@ -3331,7 +3331,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F86" s="6" t="inlineStr"/>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>La función de Maps no toma bien las direcciones</t>
+        </is>
+      </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -3349,7 +3353,7 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>App mobile nativa con Capacitor (offline first)</t>
+          <t>Modificadores por ítem en POS (extras, variantes)</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3380,7 +3384,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Notificaciones push (stock, pedidos)</t>
+          <t>App mobile nativa con Capacitor (offline first)</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -3411,7 +3415,7 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
+          <t>Notificaciones push (stock, pedidos)</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3442,7 +3446,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3462,13 +3466,44 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Roadmap v2</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr"/>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G90"/>
+  <autoFilter ref="A4:G91"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G90">
+  <conditionalFormatting sqref="A5:G91">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3480,10 +3515,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3536,7 +3571,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$90,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$91,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3551,7 +3586,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$90,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$91,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3566,7 +3601,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$90,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$91,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3581,7 +3616,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$90)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$91)</f>
         <v/>
       </c>
     </row>
@@ -3609,11 +3644,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A11,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A11,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -3624,11 +3659,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A12,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A12,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -3639,11 +3674,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A13,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A13,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -3654,11 +3689,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A14,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A14,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -3669,11 +3704,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A15,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A15,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -3684,11 +3719,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A16,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A16,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -3699,11 +3734,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A17,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A17,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -3714,11 +3749,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A18,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A18,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -3729,11 +3764,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A19,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A19,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -3744,11 +3779,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A20,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A20,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -3759,11 +3794,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A21,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A21,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -3774,11 +3809,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A22,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A22,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -3789,11 +3824,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A23,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A23,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -3804,11 +3839,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A24,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A24,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -3819,11 +3854,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A25,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A25,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -3834,11 +3869,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A26,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A26,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -3849,11 +3884,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A27,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A27,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -3864,11 +3899,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A28,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A28,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A28)-B28</f>
         <v/>
       </c>
     </row>
@@ -3879,11 +3914,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A29,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A29,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A29)-B29</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A29)-B29</f>
         <v/>
       </c>
     </row>
@@ -3894,11 +3929,11 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A30,Roadmap!$E$5:$E$90,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A30,Roadmap!$E$5:$E$91,"Hecho")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$90,A30)-B30</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$91,A30)-B30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: Gesto Servicios (boletas + form simplificado) = Hecho
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -3293,12 +3293,12 @@
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Formulario de presupuesto SIMPLIFICADO (hecho: cliente unificado, mano de obra directa, opciones plegables); boletas = comprobante de cobro no fiscal (al cobrar un presupuesto + boleta directa) en curso</t>
+          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Pendiente menor: seguir puliendo UI</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">

</xml_diff>

<commit_message>
roadmap: legal sin datos fiscales (Faro Sistemas) + pendiente "emitir recibo"
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -2435,7 +2435,7 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox de aceptación en signup. Responsable: Faro Sistemas (nombre comercial de Tomás de Sousa, persona física). FALTA: completar placeholders [CUIT/domicilio/email/jurisdicción] + revisión de un abogado</t>
+          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox en signup. Prestador: Faro Sistemas (SIN datos fiscales por etapa pre-formalización; único contacto = email en constante CONTACTO_EMAIL, hoy el gmail). AL FORMALIZAR: cargar CUIT + domicilio + jurisdicción y que un abogado revise</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -3298,7 +3298,7 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Pendiente menor: seguir puliendo UI</t>
+          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Pendiente menor: botón 'Emitir recibo' desde un presupuesto ya cobrado + seguir puliendo UI</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">

</xml_diff>

<commit_message>
roadmap: suma nomenclatura "versión" (Hecho) y afina baja de suscripción
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2074,20 +2074,24 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Dark / light toggle</t>
+          <t>Nomenclatura: los modos se presentan como 'versión' al usuario (Market, Servicios, etc.)</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Landing (switcher, precios, cierre) + /planes + confirmación de transferencia; se usan los nombres reales de los planes (Market, no inventados como 'Kiosco')</t>
+        </is>
+      </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2100,29 +2104,25 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Negocio SaaS</t>
+          <t>UX / Diseño</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>4 planes + Mercado Pago preapproval + webhook activación/suspensión</t>
+          <t>Dark / light toggle</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>src/lib/planes.ts</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Cobro por transferencia (panel admin + aviso cliente + comprobante por email)</t>
+          <t>4 planes + Mercado Pago preapproval + webhook activación/suspensión</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>Activación manual 1-click; /admin/suscripciones; emails salen al cargar RESEND_API_KEY</t>
+          <t>src/lib/planes.ts</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -2175,22 +2175,22 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Cobro automático MP/Mobbex (CUIT Monotributo + cuenta)</t>
+          <t>Cobro por transferencia (panel admin + aviso cliente + comprobante por email)</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>Bloqueado: falta CUIT + cuenta. Mientras tanto se cobra por transferencia</t>
+          <t>Activación manual 1-click; /admin/suscripciones; emails salen al cargar RESEND_API_KEY</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
@@ -2210,12 +2210,12 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Panel super-admin (gestionar tenants, métricas cross-tenant)</t>
+          <t>Cobro automático MP/Mobbex (CUIT Monotributo + cuenta)</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Panel /admin/suscripciones operativo; faltan métricas cross-tenant</t>
+          <t>Bloqueado: falta CUIT + cuenta. Mientras tanto se cobra por transferencia</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -2245,22 +2245,22 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Catálogo global cross-tenant</t>
+          <t>Panel super-admin (gestionar tenants, métricas cross-tenant)</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>Necesita OK explícito antes de implementar</t>
+          <t>Panel /admin/suscripciones operativo; faltan métricas cross-tenant</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Lanzamiento (bloqueante)</t>
+          <t>Negocio SaaS</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Dominio propio (ej: usegesto.app)</t>
+          <t>Catálogo global cross-tenant</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>URL actual no es presentable</t>
+          <t>Necesita OK explícito antes de implementar</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>SMTP con Resend (invitación, bienvenida, reset con branding)</t>
+          <t>Dominio propio (ej: usegesto.app)</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>Cron listo; falta RESEND_API_KEY en Vercel (rotar la vieja)</t>
+          <t>URL actual no es presentable</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Landing page pública (adaptativa por versión + demo en vivo)</t>
+          <t>SMTP con Resend (invitación, bienvenida, reset con branding)</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -2360,12 +2360,12 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>v3 'de oficio' LIVE: switcher de versiones auto-rotativo, demo POS con ticket de papel, foto real + captura de Gesto en celular, antes/después, FAQ, pricing al MEP, paleta terracota (sin neón), responsive mobile. Login rediseñado (split de marca)</t>
+          <t>Cron listo; falta RESEND_API_KEY en Vercel (rotar la vieja)</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>PWA manifest + iconos (192/512, apple-touch-icon)</t>
+          <t>Landing page pública (adaptativa por versión + demo en vivo)</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2395,12 +2395,12 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>POS se usa en tablet/celular</t>
+          <t>v3 'de oficio' LIVE: switcher de versiones auto-rotativo, demo POS con ticket de papel, foto real + captura de Gesto en celular, antes/después, FAQ, pricing al MEP, paleta terracota (sin neón), responsive mobile. Login rediseñado (split de marca)</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Términos de servicio + Política de privacidad</t>
+          <t>PWA manifest + iconos (192/512, apple-touch-icon)</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox en signup. Prestador: Faro Sistemas (SIN datos fiscales por etapa pre-formalización; único contacto = email en constante CONTACTO_EMAIL, hoy el gmail). AL FORMALIZAR: cargar CUIT + domicilio + jurisdicción y que un abogado revise</t>
+          <t>POS se usa en tablet/celular</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
@@ -2450,17 +2450,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Calidad / Seguridad</t>
+          <t>Lanzamiento (bloqueante)</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Bugs críticos corregidos (stock al vender, numeración, loop /planes)</t>
+          <t>Términos de servicio + Política de privacidad</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -2468,7 +2468,11 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr"/>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>Páginas /legal/{terminos,privacidad,cookies,baja-de-datos} + links en footer + checkbox en signup. Prestador: Faro Sistemas (SIN datos fiscales por etapa pre-formalización; único contacto = email en constante CONTACTO_EMAIL, hoy el gmail). AL FORMALIZAR: cargar CUIT + domicilio + jurisdicción y que un abogado revise</t>
+        </is>
+      </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2486,7 +2490,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>ConfirmDialog reutilizable (reemplaza window.confirm en 9 comp.)</t>
+          <t>Bugs críticos corregidos (stock al vender, numeración, loop /planes)</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -2517,7 +2521,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Verificar firma de webhook MP</t>
+          <t>ConfirmDialog reutilizable (reemplaza window.confirm en 9 comp.)</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -2530,11 +2534,7 @@
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>Firma HMAC timing-safe + fail-closed en prod; cargar MP_WEBHOOK_SECRET en Vercel</t>
-        </is>
-      </c>
+      <c r="F63" s="6" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Auditoría de seguridad E2E + fixes (IDOR token MP, recibirPedido, escalación de rol, OAuth state, crons fail-closed, escape de emails)</t>
+          <t>Verificar firma de webhook MP</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>Guard test anti-omisión de byTenant; ver project_gesto_seguridad. RLS no protege capa app (byTenant única defensa)</t>
+          <t>Firma HMAC timing-safe + fail-closed en prod; cargar MP_WEBHOOK_SECRET en Vercel</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -2587,22 +2587,22 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Rate limiting en auth (login/signup)</t>
+          <t>Auditoría de seguridad E2E + fixes (IDOR token MP, recibirPedido, escalación de rol, OAuth state, crons fail-closed, escape de emails)</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>ej: @upstash/ratelimit</t>
+          <t>Guard test anti-omisión de byTenant; ver project_gesto_seguridad. RLS no protege capa app (byTenant única defensa)</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Tests de integración (flows de venta y producto)</t>
+          <t>Rate limiting en auth (login/signup)</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -2635,7 +2635,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr"/>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>ej: @upstash/ratelimit</t>
+        </is>
+      </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2653,7 +2657,7 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Export de datos (CSV ventas / inventario)</t>
+          <t>Tests de integración (flows de venta y producto)</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -2666,11 +2670,7 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>Que el cliente no sienta lock-in</t>
-        </is>
-      </c>
+      <c r="F67" s="6" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Facturación AFIP (Tusfacturas.app, A/B)</t>
+          <t>Export de datos (CSV ventas / inventario)</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>Bloqueante segmento servicios/mayorista</t>
+          <t>Que el cliente no sienta lock-in</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
@@ -2723,12 +2723,12 @@
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Historial de auditoría básico (quién creó/modificó)</t>
+          <t>Facturación AFIP (Tusfacturas.app, A/B)</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>Mínimo en productos y ventas</t>
+          <t>Bloqueante segmento servicios/mayorista</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -2753,17 +2753,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Legal / Fiscal</t>
+          <t>Calidad / Seguridad</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>CUIT + Monotributo (o Responsable Inscripto)</t>
+          <t>Historial de auditoría básico (quién creó/modificó)</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>Bloquea cobrar en regla; ojo el tope anual de Monotributo con ingresos SaaS recurrentes</t>
+          <t>Mínimo en productos y ventas</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
@@ -2793,12 +2793,12 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Registro de bases de datos ante la AAIP (Ley 25.326)</t>
+          <t>CUIT + Monotributo (o Responsable Inscripto)</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>Sos responsable de la PII de los clientes y de SUS clientes</t>
+          <t>Bloquea cobrar en regla; ojo el tope anual de Monotributo con ingresos SaaS recurrentes</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Botón de baja + arrepentimiento de suscripción (Res. 424/2020)</t>
+          <t>Registro de bases de datos ante la AAIP (Ley 25.326)</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>Cancelación online fácil y visible; ya existe cancelarSuscripcion</t>
+          <t>Sos responsable de la PII de los clientes y de SUS clientes</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
@@ -2863,22 +2863,22 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Cláusulas de transferencia internacional de datos</t>
+          <t>Botón de baja + arrepentimiento de suscripción (Res. 424/2020)</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>Datos en AWS us-east-1; Ley 25.326 exige resguardos (EE.UU. no es país adecuado por defecto)</t>
+          <t>Ya existe cancelarSuscripcion + página /legal/baja-de-datos que explica el proceso; falta el botón de arrepentimiento bien visible</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Estructura societaria (SAS) + acuerdo escrito con socio</t>
+          <t>Cláusulas de transferencia internacional de datos</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>Separa patrimonio del riesgo; formaliza la participación de Facu</t>
+          <t>Datos en AWS us-east-1; Ley 25.326 exige resguardos (EE.UU. no es país adecuado por defecto)</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Contrato de servicio / SLA con clientes</t>
+          <t>Estructura societaria (SAS) + acuerdo escrito con socio</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>Dueño de los datos (el cliente), uptime, soporte, límite de responsabilidad</t>
+          <t>Separa patrimonio del riesgo; formaliza la participación de Facu</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
@@ -2963,17 +2963,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Infra / Escalado</t>
+          <t>Legal / Fiscal</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Vercel Pro + Supabase Pro</t>
+          <t>Contrato de servicio / SLA con clientes</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>Vercel Hobby es no comercial; Supabase Free se pausa a los 7 días. Bloquea producción real</t>
+          <t>Dueño de los datos (el cliente), uptime, soporte, límite de responsabilidad</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -3003,12 +3003,12 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Backups diarios + PITR + probar un restore</t>
+          <t>Vercel Pro + Supabase Pro</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>Un backup sin restore probado no es un backup</t>
+          <t>Vercel Hobby es no comercial; Supabase Free se pausa a los 7 días. Bloquea producción real</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Monitoreo: activar Sentry + uptime check</t>
+          <t>Backups diarios + PITR + probar un restore</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>SENTRY_DSN ya está en el build, falta activarlo + un cron canario</t>
+          <t>Un backup sin restore probado no es un backup</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Email deliverability: dominio + SPF/DKIM/DMARC (Resend)</t>
+          <t>Monitoreo: activar Sentry + uptime check</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>Si no, comprobantes y facturas caen en spam</t>
+          <t>SENTRY_DSN ya está en el build, falta activarlo + un cron canario</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Encriptar tokens MP del negocio at-rest</t>
+          <t>Email deliverability: dominio + SPF/DKIM/DMARC (Resend)</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>Hoy en texto plano en tenants (hallazgo de seguridad #9)</t>
+          <t>Si no, comprobantes y facturas caen en spam</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -3138,12 +3138,12 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Backlog / Ideas</t>
+          <t>Infra / Escalado</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Consultor de precios para cliente final (pantalla pública con QR)</t>
+          <t>Encriptar tokens MP del negocio at-rest</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>Diferenciador único; ruta /p/[tenantSlug]</t>
+          <t>Hoy en texto plano en tenants (hallazgo de seguridad #9)</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -3173,12 +3173,12 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Versiones / Verticales</t>
+          <t>Backlog / Ideas</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Mejorar login/registro: sumarle contenido útil (hoy se siente vacío)</t>
+          <t>Consultor de precios para cliente final (pantalla pública con QR)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>Split de marca ya hecho; falta valor real que sume</t>
+          <t>Diferenciador único; ruta /p/[tenantSlug]</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
@@ -3213,22 +3213,22 @@
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Gesto Balanza funcional: integración con balanza digital + venta por peso</t>
+          <t>Mejorar login/registro: sumarle contenido útil (hoy se siente vacío)</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>Hoy figura 'próximamente'; armarla de verdad para que funcione con balanzas</t>
+          <t>Split de marca ya hecho; falta valor real que sume</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
+          <t>Gesto Balanza funcional: integración con balanza digital + venta por peso</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Hoy figura 'próximamente'</t>
+          <t>Hoy figura 'próximamente'; armarla de verdad para que funcione con balanzas</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
+          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Pendiente menor: botón 'Emitir recibo' desde un presupuesto ya cobrado + seguir puliendo UI</t>
+          <t>Hoy figura 'próximamente'</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
+          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3328,12 +3328,12 @@
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>La función de Maps no toma bien las direcciones</t>
+          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Pendiente menor: botón 'Emitir recibo' desde un presupuesto ya cobrado + seguir puliendo UI</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -3348,17 +3348,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Modificadores por ítem en POS (extras, variantes)</t>
+          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
@@ -3366,7 +3366,11 @@
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F87" s="6" t="inlineStr"/>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>La función de Maps no toma bien las direcciones</t>
+        </is>
+      </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
           <t>2026-06-21</t>
@@ -3384,7 +3388,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>App mobile nativa con Capacitor (offline first)</t>
+          <t>Modificadores por ítem en POS (extras, variantes)</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -3415,7 +3419,7 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Notificaciones push (stock, pedidos)</t>
+          <t>App mobile nativa con Capacitor (offline first)</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3446,7 +3450,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
+          <t>Notificaciones push (stock, pedidos)</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3477,7 +3481,7 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3497,13 +3501,44 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Roadmap v2</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr"/>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G91"/>
+  <autoFilter ref="A4:G92"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G91">
+  <conditionalFormatting sqref="A5:G92">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3515,10 +3550,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3571,7 +3606,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$91,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$92,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3586,7 +3621,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$91,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$92,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3601,7 +3636,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$91,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$92,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3616,7 +3651,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$91)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$92)</f>
         <v/>
       </c>
     </row>
@@ -3644,11 +3679,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A11,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A11,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -3659,11 +3694,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A12,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A12,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -3674,11 +3709,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A13,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A13,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -3689,11 +3724,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A14,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A14,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -3704,11 +3739,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A15,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A15,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -3719,11 +3754,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A16,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A16,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -3734,11 +3769,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A17,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A17,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -3749,11 +3784,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A18,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A18,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -3764,11 +3799,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A19,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A19,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -3779,11 +3814,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A20,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A20,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -3794,11 +3829,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A21,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A21,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -3809,11 +3844,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A22,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A22,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -3824,11 +3859,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A23,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A23,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -3839,11 +3874,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A24,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A24,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -3854,11 +3889,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A25,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A25,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -3869,11 +3904,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A26,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A26,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -3884,11 +3919,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A27,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A27,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -3899,11 +3934,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A28,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A28,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A28)-B28</f>
         <v/>
       </c>
     </row>
@@ -3914,11 +3949,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A29,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A29,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A29)-B29</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A29)-B29</f>
         <v/>
       </c>
     </row>
@@ -3929,11 +3964,11 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A30,Roadmap!$E$5:$E$91,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A30,Roadmap!$E$5:$E$92,"Hecho")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$91,A30)-B30</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$92,A30)-B30</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: Atmosféricos agenda+futuros hecho, falta Maps
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -3363,12 +3363,12 @@
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>La función de Maps no toma bien las direcciones</t>
+          <t>Historial ya existía; AGENDA (navegación entre días) + pedidos para días futuros HECHO. FALTA: arreglar la ruta en Maps (geocoding de direcciones de texto falla; evaluar guardar ubicación exacta / link de Maps por pedido sin pagar Google API)</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">

</xml_diff>

<commit_message>
roadmap: Atmosféricos = Hecho (Maps arreglado)
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -3363,12 +3363,12 @@
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>Historial ya existía; AGENDA (navegación entre días) + pedidos para días futuros HECHO. FALTA: arreglar la ruta en Maps (geocoding de direcciones de texto falla; evaluar guardar ubicación exacta / link de Maps por pedido sin pagar Google API)</t>
+          <t>Historial ya existía; AGENDA (navegación entre días) + pedidos para días futuros HECHO. Maps ARREGLADO: campo 'ubicación exacta' (link de Maps) por pedido; geo.ts extrae coordenadas del link y la ruta usa el punto exacto en vez del texto. Migración 0010 en dev+prod</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">

</xml_diff>

<commit_message>
roadmap: login a fondo = Hecho
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -3223,12 +3223,12 @@
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>Split de marca ya hecho; falta valor real que sume</t>
+          <t>Split de marca + recuperación de contraseña ya estaban. Sumado: ver/ocultar contraseña (PasswordInput) en login/signup/reset, errores específicos (email sin confirmar, rate-limit, email ya registrado), pie con Términos/Privacidad/ayuda por mail, indicador de fuerza de contraseña</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">

</xml_diff>

<commit_message>
roadmap: Balanza = Hecho (venta por peso)
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -3258,12 +3258,12 @@
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>Hoy figura 'próximamente'; armarla de verdad para que funcione con balanzas</t>
+          <t>POS con venta por peso: modal de gramos (atajos 250/500/1000 g + subtotal en vivo), edición de peso en carrito, y lectura de etiquetas de balanza con peso embebido (EAN-13 prefijo 2 -&gt; PLU + peso). Página /dashboard/balanza con guía de 3 pasos. Plan habilitado (proximamente:false) y nav activo. Pendiente futuro: configurar el formato exacto de etiqueta por marca de balanza</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">

</xml_diff>

<commit_message>
roadmap: sección Marketing/Conversión (wizard+WhatsApp hechos, pendientes del análisis)
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SaaS de gestión comercial multi-tenant · Actualizado 2026-06-21 · Editá la columna Estado y la fecha al cerrar cada tarea</t>
+          <t>SaaS de gestión comercial multi-tenant · Actualizado 2026-06-22 · Editá la columna Estado y la fecha al cerrar cada tarea</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       <c r="F21" s="6" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       <c r="F28" s="6" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       <c r="F30" s="6" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       <c r="F31" s="6" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       <c r="F38" s="6" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       <c r="F40" s="6" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       <c r="F41" s="6" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       <c r="F42" s="6" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       <c r="F43" s="6" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       <c r="F44" s="6" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       <c r="F46" s="6" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       <c r="F47" s="6" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
       <c r="F48" s="6" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       <c r="F49" s="6" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
       <c r="F51" s="6" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2506,7 @@
       <c r="F62" s="6" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       <c r="F63" s="6" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       <c r="F67" s="6" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       <c r="F88" s="6" t="inlineStr"/>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       <c r="F89" s="6" t="inlineStr"/>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       <c r="F90" s="6" t="inlineStr"/>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3497,7 @@
       <c r="F91" s="6" t="inlineStr"/>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3528,17 +3528,332 @@
       <c r="F92" s="6" t="inlineStr"/>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>Registro en mini-wizard modal (versión -&gt; cuenta), sin mandar al login frío</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>Modal in-page (no popup) que abren los CTA 'Empezá gratis'. Paso 1 elegís versión, paso 2 creás cuenta; la versión se hereda al onboarding</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>Login con Google (OAuth)</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>En progreso</t>
+        </is>
+      </c>
+      <c r="F94" s="6" t="inlineStr">
+        <is>
+          <t>Código cableado en el wizard y disponible. FALTA: habilitar el provider Google en Supabase (Auth -&gt; Providers) con credenciales de Google Cloud Console</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Botón de WhatsApp flotante en la landing</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>Sugerido por Deepseek y Gemini. FALTA: reemplazar el número placeholder por el real</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>Landing pages por vertical (/market, /atmosfericos, /balanza) para pauta en Meta Ads</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>Gemini: la página de destino tiene que hablarle solo a ese rubro para no diluir la conversión</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>Dominio propio (ej. gesto.com.ar) apuntado en Vercel</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
+        <is>
+          <t>Gemini: faro-sistemas.vercel.app no transmite 'Gesto' y resta confianza</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>Nav de la landing con Versiones y Ayuda (hoy solo Precios)</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>Deepseek</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="n">
+        <v>95</v>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>Sello 'datos encriptados' + destacar '14 días sin tarjeta' como badge</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>Deepseek: confianza sin necesitar testimonios</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>Testimonios / casos de éxito</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
+        <is>
+          <t>Dejar el espacio diseñado y llenarlo con los primeros clientes reales (no inventar)</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>Decidir precio en ARS prominente y USD como referencia</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>Deepseek; toca la decisión de negocio de cobro al MEP en USD</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G92"/>
+  <autoFilter ref="A4:G101"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G92">
+  <conditionalFormatting sqref="A5:G101">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3550,10 +3865,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3567,7 +3882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3606,7 +3921,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$92,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$101,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3621,7 +3936,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$92,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$101,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3636,7 +3951,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$92,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$101,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3651,7 +3966,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$92)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$101)</f>
         <v/>
       </c>
     </row>
@@ -3679,11 +3994,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A11,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A11,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -3694,11 +4009,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A12,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A12,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -3709,11 +4024,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A13,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A13,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -3724,11 +4039,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A14,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A14,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -3739,11 +4054,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A15,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A15,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -3754,11 +4069,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A16,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A16,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -3769,11 +4084,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A17,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A17,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -3784,11 +4099,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A18,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A18,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -3799,11 +4114,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A19,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A19,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -3814,11 +4129,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A20,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A20,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -3829,11 +4144,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A21,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A21,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -3844,11 +4159,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A22,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A22,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -3859,11 +4174,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A23,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A23,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -3874,11 +4189,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A24,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A24,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -3889,11 +4204,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A25,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A25,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -3904,11 +4219,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A26,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A26,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -3919,11 +4234,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A27,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A27,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -3934,11 +4249,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A28,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A28,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A28)-B28</f>
         <v/>
       </c>
     </row>
@@ -3949,11 +4264,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A29,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A29,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A29)-B29</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A29)-B29</f>
         <v/>
       </c>
     </row>
@@ -3964,11 +4279,26 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A30,Roadmap!$E$5:$E$92,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A30,Roadmap!$E$5:$E$101,"Hecho")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$92,A30)-B30</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A30)-B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A31,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <v/>
+      </c>
+      <c r="C31">
+        <f>COUNTIFS(Roadmap!$B$5:$B$101,A31)-B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: CTA por versión, sellos, nav y ARS = Hecho
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3728,12 +3728,12 @@
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>Deepseek</t>
+          <t>Nav: 'Versiones' (antes 'Cómo funciona') + 'Ayuda' al WhatsApp</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Sello 'datos encriptados' + destacar '14 días sin tarjeta' como badge</t>
+          <t>CTA por versión en precios (abre el wizard con esa versión)</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -3763,12 +3763,12 @@
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>Deepseek: confianza sin necesitar testimonios</t>
+          <t>Cada tarjeta: 'Probar [versión] gratis' -&gt; abre el wizard con esa versión preelegida</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Testimonios / casos de éxito</t>
+          <t>Precio en ARS más visible (manteniendo USD como principal)</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -3798,12 +3798,12 @@
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>Dejar el espacio diseñado y llenarlo con los primeros clientes reales (no inventar)</t>
+          <t>El ARS se agrandó (16px, seminegrita); el USD sigue siendo el número grande. Se mantiene el cobro al MEP en USD</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Decidir precio en ARS prominente y USD como referencia</t>
+          <t>Sello 'datos encriptados' + destacar '14 días sin tarjeta' como badge</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -3833,27 +3833,62 @@
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
+        <is>
+          <t>Sellos bajo los planes: datos encriptados (SSL), 14 días sin tarjeta, cancelás cuando quieras</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>Testimonios / casos de éxito</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="inlineStr">
+        <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>Deepseek; toca la decisión de negocio de cobro al MEP en USD</t>
-        </is>
-      </c>
-      <c r="G101" s="5" t="inlineStr">
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>Dejar el espacio diseñado y llenarlo con los primeros clientes reales (no inventar)</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G101"/>
+  <autoFilter ref="A4:G102"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G101">
+  <conditionalFormatting sqref="A5:G102">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3865,10 +3900,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3921,7 +3956,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$101,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$102,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3936,7 +3971,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$101,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$102,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3951,7 +3986,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$101,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$102,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -3966,7 +4001,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$101)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$102)</f>
         <v/>
       </c>
     </row>
@@ -3994,11 +4029,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A11,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A11,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -4009,11 +4044,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A12,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A12,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -4024,11 +4059,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A13,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A13,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -4039,11 +4074,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A14,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A14,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -4054,11 +4089,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A15,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A15,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -4069,11 +4104,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A16,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A16,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -4084,11 +4119,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A17,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A17,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -4099,11 +4134,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A18,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A18,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -4114,11 +4149,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A19,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A19,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -4129,11 +4164,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A20,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A20,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -4144,11 +4179,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A21,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A21,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -4159,11 +4194,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A22,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A22,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -4174,11 +4209,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A23,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A23,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -4189,11 +4224,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A24,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A24,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -4204,11 +4239,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A25,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A25,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -4219,11 +4254,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A26,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A26,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -4234,11 +4269,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A27,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A27,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -4249,11 +4284,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A28,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A28,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A28)-B28</f>
         <v/>
       </c>
     </row>
@@ -4264,11 +4299,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A29,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A29,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A29)-B29</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A29)-B29</f>
         <v/>
       </c>
     </row>
@@ -4279,11 +4314,11 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A30,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A30,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A30)-B30</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A30)-B30</f>
         <v/>
       </c>
     </row>
@@ -4294,11 +4329,11 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A31,Roadmap!$E$5:$E$101,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A31,Roadmap!$E$5:$E$102,"Hecho")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS(Roadmap!$B$5:$B$101,A31)-B31</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$102,A31)-B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: impresión térmica BT/USB hecha + balanza portada al POS real
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>POS con venta por peso: modal de gramos (atajos 250/500/1000 g + subtotal en vivo), edición de peso en carrito, y lectura de etiquetas de balanza con peso embebido (EAN-13 prefijo 2 -&gt; PLU + peso). Página /dashboard/balanza con guía de 3 pasos. Plan habilitado (proximamente:false) y nav activo. Pendiente futuro: configurar el formato exacto de etiqueta por marca de balanza</t>
+          <t>Plan habilitado + nav + página guía /dashboard/balanza. Lectura de etiquetas de balanza con peso embebido (EAN-13 prefijo 2 -&gt; PLU + peso) PORTADA al POS real (pos-container; el primer intento quedó en un componente muerto ya borrado). Peso a mano: por ahora vía 'línea suelta'. Pendiente futuro: modal de peso al tocar un producto por_kg, y configurar el formato exacto de etiqueta por marca de balanza</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -3278,12 +3278,12 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Versiones / Verticales</t>
+          <t>POS / Hardware</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
+          <t>Impresión de tickets: térmica directa por Bluetooth y USB (ESC/POS)</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>Hoy figura 'próximamente'</t>
+          <t>Motor ESC/POS (CP850), transporte Web Bluetooth + WebUSB, botón 'Térmica' en el modal post-venta que conecta la ticketera e imprime de un toque. window.print() (sistema/AirPrint) y PDF ya existían. iOS solo por window.print(). Pendiente futuro: impresoras WiFi por IP (puerto 9100) requieren un puente/print-server o ePOS HTTP; app nativa abriría todo</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
+          <t>Gesto Food: POS propio (comandas, mesas, cocina/KDS) — muy distinto a Market</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -3328,12 +3328,12 @@
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Botón 'Emitir recibo' desde un presupuesto cobrado HECHO (PDF como recibo, sin duplicar ingreso). Pendiente menor: seguir puliendo UI</t>
+          <t>Hoy figura 'próximamente'</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
+          <t>Gesto Servicios: emitir boletas además de presupuestos + simplificar botones/UI</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>Historial ya existía; AGENDA (navegación entre días) + pedidos para días futuros HECHO. Maps ARREGLADO: campo 'ubicación exacta' (link de Maps) por pedido; geo.ts extrae coordenadas del link y la ruta usa el punto exacto en vez del texto. Migración 0010 en dev+prod</t>
+          <t>Form de presupuesto simplificado + BOLETAS de punta a punta: boleta directa (form modo boleta con método de pago), numeración propia, lista /dashboard/boletas + nav, detalle adaptado y PDF como RECIBO. Migración 0009 aplicada en dev+prod. Comprobante NO fiscal. Botón 'Emitir recibo' desde un presupuesto cobrado HECHO (PDF como recibo, sin duplicar ingreso). Pendiente menor: seguir puliendo UI</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
@@ -3383,25 +3383,29 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>Versiones / Verticales</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Modificadores por ítem en POS (extras, variantes)</t>
+          <t>Gesto Atmosféricos: historial, agenda y pedidos para días futuros + arreglar ruta en Maps</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="F88" s="6" t="inlineStr"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>Historial ya existía; AGENDA (navegación entre días) + pedidos para días futuros HECHO. Maps ARREGLADO: campo 'ubicación exacta' (link de Maps) por pedido; geo.ts extrae coordenadas del link y la ruta usa el punto exacto en vez del texto. Migración 0010 en dev+prod</t>
+        </is>
+      </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
@@ -3419,7 +3423,7 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>App mobile nativa con Capacitor (offline first)</t>
+          <t>Modificadores por ítem en POS (extras, variantes)</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -3450,7 +3454,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Notificaciones push (stock, pedidos)</t>
+          <t>App mobile nativa con Capacitor (offline first)</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -3481,7 +3485,7 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
+          <t>Notificaciones push (stock, pedidos)</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -3512,7 +3516,7 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
+          <t>Dashboard financiero avanzado (márgenes, rentabilidad)</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -3538,29 +3542,25 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>Marketing / Conversión</t>
+          <t>Roadmap v2</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Registro en mini-wizard modal (versión -&gt; cuenta), sin mandar al login frío</t>
+          <t>Multi-sucursal (varios locales bajo una cuenta madre)</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="F93" s="6" t="inlineStr">
-        <is>
-          <t>Modal in-page (no popup) que abren los CTA 'Empezá gratis'. Paso 1 elegís versión, paso 2 creás cuenta; la versión se hereda al onboarding</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr"/>
       <c r="G93" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Login con Google (OAuth)</t>
+          <t>Registro en mini-wizard modal (versión -&gt; cuenta), sin mandar al login frío</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -3588,12 +3588,12 @@
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>En progreso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>Código cableado en el wizard y disponible. FALTA: habilitar el provider Google en Supabase (Auth -&gt; Providers) con credenciales de Google Cloud Console</t>
+          <t>Modal in-page (no popup) que abren los CTA 'Empezá gratis'. Paso 1 elegís versión, paso 2 creás cuenta; la versión se hereda al onboarding</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Botón de WhatsApp flotante en la landing</t>
+          <t>Login con Google (OAuth)</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -3623,12 +3623,12 @@
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>En progreso</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>Sugerido por Deepseek y Gemini. Número real cargado (wa.me/5491166644837), mensaje pre-cargado</t>
+          <t>Código cableado en el wizard y disponible. FALTA: habilitar el provider Google en Supabase (Auth -&gt; Providers) con credenciales de Google Cloud Console</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Landing pages por vertical (/market, /atmosfericos, /balanza) para pauta en Meta Ads</t>
+          <t>Botón de WhatsApp flotante en la landing</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -3658,12 +3658,12 @@
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>Gemini: la página de destino tiene que hablarle solo a ese rubro para no diluir la conversión</t>
+          <t>Sugerido por Deepseek y Gemini. Número real cargado (wa.me/5491166644837), mensaje pre-cargado</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Dominio propio (ej. gesto.com.ar) apuntado en Vercel</t>
+          <t>Landing pages por vertical (/market, /atmosfericos, /balanza) para pauta en Meta Ads</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -3698,7 +3698,7 @@
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>Gemini: faro-sistemas.vercel.app no transmite 'Gesto' y resta confianza</t>
+          <t>Gemini: la página de destino tiene que hablarle solo a ese rubro para no diluir la conversión</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
@@ -3718,22 +3718,22 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Nav de la landing con Versiones y Ayuda (hoy solo Precios)</t>
+          <t>Dominio propio (ej. gesto.com.ar) apuntado en Vercel</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>Nav: 'Versiones' (antes 'Cómo funciona') + 'Ayuda' al WhatsApp</t>
+          <t>Gemini: faro-sistemas.vercel.app no transmite 'Gesto' y resta confianza</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>CTA por versión en precios (abre el wizard con esa versión)</t>
+          <t>Nav de la landing con Versiones y Ayuda (hoy solo Precios)</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>Cada tarjeta: 'Probar [versión] gratis' -&gt; abre el wizard con esa versión preelegida</t>
+          <t>Nav: 'Versiones' (antes 'Cómo funciona') + 'Ayuda' al WhatsApp</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -3788,7 +3788,7 @@
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Precio en ARS más visible (manteniendo USD como principal)</t>
+          <t>CTA por versión en precios (abre el wizard con esa versión)</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>El ARS se agrandó (16px, seminegrita); el USD sigue siendo el número grande. Se mantiene el cobro al MEP en USD</t>
+          <t>Cada tarjeta: 'Probar [versión] gratis' -&gt; abre el wizard con esa versión preelegida</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Sello 'datos encriptados' + destacar '14 días sin tarjeta' como badge</t>
+          <t>Precio en ARS más visible (manteniendo USD como principal)</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>Sellos bajo los planes: datos encriptados (SSL), 14 días sin tarjeta, cancelás cuando quieras</t>
+          <t>El ARS se agrandó (16px, seminegrita); el USD sigue siendo el número grande. Se mantiene el cobro al MEP en USD</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
@@ -3858,37 +3858,72 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
+          <t>Sello 'datos encriptados' + destacar '14 días sin tarjeta' como badge</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>Sellos bajo los planes: datos encriptados (SSL), 14 días sin tarjeta, cancelás cuando quieras</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Marketing / Conversión</t>
+        </is>
+      </c>
+      <c r="C103" s="6" t="inlineStr">
+        <is>
           <t>Testimonios / casos de éxito</t>
         </is>
       </c>
-      <c r="D102" s="4" t="inlineStr">
+      <c r="D103" s="4" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="E102" s="7" t="inlineStr">
+      <c r="E103" s="7" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="F102" s="6" t="inlineStr">
+      <c r="F103" s="6" t="inlineStr">
         <is>
           <t>Dejar el espacio diseñado y llenarlo con los primeros clientes reales (no inventar)</t>
         </is>
       </c>
-      <c r="G102" s="5" t="inlineStr">
+      <c r="G103" s="5" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G102"/>
+  <autoFilter ref="A4:G103"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G102">
+  <conditionalFormatting sqref="A5:G103">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3900,10 +3935,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3917,7 +3952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3956,7 +3991,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$102,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$103,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -3971,7 +4006,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$102,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$103,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -3986,7 +4021,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$102,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$103,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -4001,7 +4036,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$102)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$103)</f>
         <v/>
       </c>
     </row>
@@ -4029,11 +4064,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A11,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A11,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -4044,11 +4079,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A12,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A12,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -4059,11 +4094,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A13,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A13,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -4074,11 +4109,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A14,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A14,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -4089,11 +4124,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A15,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A15,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -4104,11 +4139,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A16,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A16,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -4119,11 +4154,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A17,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A17,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -4134,11 +4169,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A18,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A18,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -4149,11 +4184,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A19,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A19,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -4164,11 +4199,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A20,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A20,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -4179,11 +4214,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A21,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A21,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -4194,11 +4229,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A22,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A22,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -4209,11 +4244,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A23,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A23,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -4224,11 +4259,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A24,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A24,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -4239,11 +4274,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A25,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A25,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -4254,11 +4289,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A26,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A26,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -4269,11 +4304,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A27,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A27,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -4284,11 +4319,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A28,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A28,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A28)-B28</f>
         <v/>
       </c>
     </row>
@@ -4299,41 +4334,56 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A29,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A29,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A29)-B29</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A29)-B29</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Roadmap v2</t>
+          <t>POS / Hardware</t>
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A30,Roadmap!$E$5:$E$102,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A30,Roadmap!$E$5:$E$103,"Hecho")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A30)-B30</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A30)-B30</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Roadmap v2</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A31,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <v/>
+      </c>
+      <c r="C31">
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A31)-B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Marketing / Conversión</t>
         </is>
       </c>
-      <c r="B31">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A31,Roadmap!$E$5:$E$102,"Hecho")</f>
-        <v/>
-      </c>
-      <c r="C31">
-        <f>COUNTIFS(Roadmap!$B$5:$B$102,A31)-B31</f>
+      <c r="B32">
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A32,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <v/>
+      </c>
+      <c r="C32">
+        <f>COUNTIFS(Roadmap!$B$5:$B$103,A32)-B32</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
roadmap: bloque "QA por planes (jun-2026)" + MP
Agrega las 23 tareas del QA por planes + las 2 de MercadoPago (conectar = Hecho,
cobro real por API = Pendiente). Actualiza fecha a 2026-06-25.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roadmap-gesto.xlsx
+++ b/roadmap-gesto.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$4:$G$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SaaS de gestión comercial multi-tenant · Actualizado 2026-06-22 · Editá la columna Estado y la fecha al cerrar cada tarea</t>
+          <t>SaaS de gestión comercial multi-tenant · Actualizado 2026-06-25 · Editá la columna Estado y la fecha al cerrar cada tarea</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       <c r="F5" s="6" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -937,7 +937,7 @@
       <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       <c r="F20" s="6" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
       <c r="F21" s="6" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       <c r="F28" s="6" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       <c r="F30" s="6" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       <c r="F31" s="6" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       <c r="F38" s="6" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       <c r="F40" s="6" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       <c r="F41" s="6" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       <c r="F42" s="6" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       <c r="F43" s="6" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1900,7 +1900,7 @@
       <c r="F44" s="6" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       <c r="F46" s="6" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1997,7 @@
       <c r="F47" s="6" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
       <c r="F48" s="6" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       <c r="F49" s="6" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
       <c r="F51" s="6" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2506,7 @@
       <c r="F62" s="6" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       <c r="F63" s="6" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       <c r="F67" s="6" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
       <c r="F89" s="6" t="inlineStr"/>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       <c r="F90" s="6" t="inlineStr"/>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       <c r="F91" s="6" t="inlineStr"/>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       <c r="F92" s="6" t="inlineStr"/>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       <c r="F93" s="6" t="inlineStr"/>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -3913,17 +3913,841 @@
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C104" s="6" t="inlineStr">
+        <is>
+          <t>MP: conectar cuenta del negocio (OAuth) — arreglado, conecta en prod</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F104" s="6" t="inlineStr">
+        <is>
+          <t>Faltaban MP_APP_ID/MP_CLIENT_SECRET en Vercel + redirect_uri canónico. Se fijó NEXT_PUBLIC_APP_URL=faro-sistemas (eliminado el fallback -gold) y mp-url usa getAppUrl(). Callback con diagnóstico ?reason=. Cuenta de prueba conectó OK (ID 642364293)</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="4" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>Cobro REAL por Mercado Pago (QR dinámico / link / Point) con la cuenta conectada</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F105" s="6" t="inlineStr">
+        <is>
+          <t>HOY 'Mercado Pago' en el POS solo MARCA la venta como pagada (registro manual). getMPNegocioToken existe pero NO se usa. Falta: crear QR/orden por API de MP + webhook de confirmación que marque la venta cobrada</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C106" s="6" t="inlineStr">
+        <is>
+          <t>Nav: 'Equipo' ya no marca también 'Configuración'</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>match por href más específico. En staging, falta merge a prod</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>Nav PC: sacar el desplegable 'Más', listar todos los items directos</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>POS: el hint 'escribí para buscar o elegí categoría' desaparece al enfocar el buscador</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>POS: cambiar cantidad en el carrito suena igual que agregar producto</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="n">
+        <v>106</v>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>POS: sonido de agregar más contundente (~1.4x, beepAgregar)</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>POS: código de barras del buscador más grande/legible</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="n">
+        <v>108</v>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>POS: fix ticket en blanco al imprimir (Market)</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>El ticket print-only vivía dentro de un contenedor .screen-only (display:none al imprimir); ahora va por portal a document.body. PDF ya andaba. staging</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="n">
+        <v>109</v>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>Productos: stock muestra '6' no '6,000' (limpia ceros de relleno de Postgres)</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>Carga rápida: agregar campo de stock inicial (con navegación por Enter)</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>staging</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="n">
+        <v>111</v>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C115" s="6" t="inlineStr">
+        <is>
+          <t>Ticket de cuenta corriente con resumen del saldo del cliente</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F115" s="6" t="inlineStr"/>
+      <c r="G115" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>Selector de tamaño de fuente global (accesibilidad, preview en vivo)</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>Para gente que ve poco. Seleccionable al inicio/onboarding + en config</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="n">
+        <v>113</v>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C117" s="6" t="inlineStr">
+        <is>
+          <t>Eliminar grupos de variantes — dejar solo categorías (el buscador ya cubre)</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>DESTRUCTIVA: migración de DB. Reemplaza la entrada 'Grupos de variantes'. Revisar impacto en plan balanza</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="n">
+        <v>114</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr">
+        <is>
+          <t>Probar importación CSV (generar un CSV de ejemplo y validar)</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F118" s="6" t="inlineStr"/>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>Filtros en el historial (por fecha, cliente, etc.)</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>Hoy solo filtra por período</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C120" s="6" t="inlineStr">
+        <is>
+          <t>Cliente: al seleccionarlo ver su ficha (datos/historial/saldo), no el form de edición; botón 'Editar' aparte</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F120" s="6" t="inlineStr"/>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C121" s="6" t="inlineStr">
+        <is>
+          <t>Reportes: al cambiar el período recalcular TODOS los datos, no solo el gráfico</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F121" s="6" t="inlineStr">
+        <is>
+          <t>Verificar; con pocas ventas en demo puede ocultarse</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>CC: aclarar/mejorar UX de 'no permitir saldo negativo'</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>El usuario no entiende cómo se maneja hoy</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="n">
+        <v>119</v>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>Proveedor: revisar selector de bandera de país (no se ve al crear)</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E123" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F123" s="6" t="inlineStr">
+        <is>
+          <t>Decidir si va y por qué</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>Botón 'generar pedido' desde Proveedor y desde Pedidos</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
+        <is>
+          <t>Hoy no hay forma de armar el pedido a proveedor</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>Categorías de gastos faltan en plan Market (revisar todos los planes)</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E125" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr"/>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>Balance mensual IA automático (cron fin de mes / fecha configurable), sin botón manual</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
+        <is>
+          <t>Opción: último día hábil del mes o fecha elegida</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>Permisos granulares por usuario (capacidades sobre el rol empleado)</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
+        <is>
+          <t>users_tenants.permisos ya existe pero sin uso. Modelo elegido: toggles por capacidad (POS, Productos, Clientes, Reportes, Gastos, etc.)</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G103"/>
+  <autoFilter ref="A4:G127"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G103">
+  <conditionalFormatting sqref="A5:G127">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="Hecho"</formula>
     </cfRule>
@@ -3935,10 +4759,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E5:E103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En progreso,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja,—"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3952,7 +4776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3991,7 +4815,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Roadmap!$E$5:$E$103,A4)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$127,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11">
@@ -4006,7 +4830,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Roadmap!$E$5:$E$103,A5)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$127,A5)</f>
         <v/>
       </c>
       <c r="C5" s="11">
@@ -4021,7 +4845,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Roadmap!$E$5:$E$103,A6)</f>
+        <f>COUNTIF(Roadmap!$E$5:$E$127,A6)</f>
         <v/>
       </c>
       <c r="C6" s="11">
@@ -4036,7 +4860,7 @@
         </is>
       </c>
       <c r="B7" s="14">
-        <f>COUNTA(Roadmap!$E$5:$E$103)</f>
+        <f>COUNTA(Roadmap!$E$5:$E$127)</f>
         <v/>
       </c>
     </row>
@@ -4064,11 +4888,11 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A11,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A11,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A11)-B11</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A11)-B11</f>
         <v/>
       </c>
     </row>
@@ -4079,11 +4903,11 @@
         </is>
       </c>
       <c r="B12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A12,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A12,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A12)-B12</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A12)-B12</f>
         <v/>
       </c>
     </row>
@@ -4094,11 +4918,11 @@
         </is>
       </c>
       <c r="B13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A13,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A13,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A13)-B13</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A13)-B13</f>
         <v/>
       </c>
     </row>
@@ -4109,11 +4933,11 @@
         </is>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A14,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A14,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A14)-B14</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A14)-B14</f>
         <v/>
       </c>
     </row>
@@ -4124,11 +4948,11 @@
         </is>
       </c>
       <c r="B15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A15,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A15,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A15)-B15</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A15)-B15</f>
         <v/>
       </c>
     </row>
@@ -4139,11 +4963,11 @@
         </is>
       </c>
       <c r="B16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A16,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A16,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A16)-B16</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A16)-B16</f>
         <v/>
       </c>
     </row>
@@ -4154,11 +4978,11 @@
         </is>
       </c>
       <c r="B17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A17,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A17,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A17)-B17</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A17)-B17</f>
         <v/>
       </c>
     </row>
@@ -4169,11 +4993,11 @@
         </is>
       </c>
       <c r="B18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A18,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A18,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A18)-B18</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A18)-B18</f>
         <v/>
       </c>
     </row>
@@ -4184,11 +5008,11 @@
         </is>
       </c>
       <c r="B19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A19,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A19,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A19)-B19</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A19)-B19</f>
         <v/>
       </c>
     </row>
@@ -4199,11 +5023,11 @@
         </is>
       </c>
       <c r="B20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A20,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A20,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A20)-B20</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A20)-B20</f>
         <v/>
       </c>
     </row>
@@ -4214,11 +5038,11 @@
         </is>
       </c>
       <c r="B21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A21,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A21,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A21)-B21</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A21)-B21</f>
         <v/>
       </c>
     </row>
@@ -4229,11 +5053,11 @@
         </is>
       </c>
       <c r="B22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A22,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A22,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A22)-B22</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A22)-B22</f>
         <v/>
       </c>
     </row>
@@ -4244,11 +5068,11 @@
         </is>
       </c>
       <c r="B23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A23,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A23,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A23)-B23</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A23)-B23</f>
         <v/>
       </c>
     </row>
@@ -4259,11 +5083,11 @@
         </is>
       </c>
       <c r="B24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A24,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A24,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A24)-B24</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A24)-B24</f>
         <v/>
       </c>
     </row>
@@ -4274,11 +5098,11 @@
         </is>
       </c>
       <c r="B25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A25,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A25,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A25)-B25</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A25)-B25</f>
         <v/>
       </c>
     </row>
@@ -4289,11 +5113,11 @@
         </is>
       </c>
       <c r="B26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A26,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A26,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C26">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A26)-B26</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A26)-B26</f>
         <v/>
       </c>
     </row>
@@ -4304,11 +5128,11 @@
         </is>
       </c>
       <c r="B27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A27,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A27,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A27)-B27</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A27)-B27</f>
         <v/>
       </c>
     </row>
@@ -4319,11 +5143,11 @@
         </is>
       </c>
       <c r="B28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A28,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A28,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C28">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A28)-B28</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A28)-B28</f>
         <v/>
       </c>
     </row>
@@ -4334,11 +5158,11 @@
         </is>
       </c>
       <c r="B29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A29,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A29,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C29">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A29)-B29</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A29)-B29</f>
         <v/>
       </c>
     </row>
@@ -4349,11 +5173,11 @@
         </is>
       </c>
       <c r="B30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A30,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A30,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C30">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A30)-B30</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A30)-B30</f>
         <v/>
       </c>
     </row>
@@ -4364,11 +5188,11 @@
         </is>
       </c>
       <c r="B31">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A31,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A31,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C31">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A31)-B31</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A31)-B31</f>
         <v/>
       </c>
     </row>
@@ -4379,11 +5203,26 @@
         </is>
       </c>
       <c r="B32">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A32,Roadmap!$E$5:$E$103,"Hecho")</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A32,Roadmap!$E$5:$E$127,"Hecho")</f>
         <v/>
       </c>
       <c r="C32">
-        <f>COUNTIFS(Roadmap!$B$5:$B$103,A32)-B32</f>
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A32)-B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>QA por planes (jun-2026)</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A33,Roadmap!$E$5:$E$127,"Hecho")</f>
+        <v/>
+      </c>
+      <c r="C33">
+        <f>COUNTIFS(Roadmap!$B$5:$B$127,A33)-B33</f>
         <v/>
       </c>
     </row>

</xml_diff>